<commit_message>
Refactor hierarchy importer to enforce prepared parent locations and opaque rack names
Update the hierarchy importer to require existing site and parent location slugs, ensuring only direct child locations and racks are created. Revise rack naming to accept opaque names without parsing for delimiters, enhancing flexibility in naming conventions. Update documentation to reflect these changes, including operator runbook and requirements adjustments, ensuring clarity on the new import process and slug management.
</commit_message>
<xml_diff>
--- a/samples/1_hierarchy_invalid.xlsx
+++ b/samples/1_hierarchy_invalid.xlsx
@@ -417,80 +417,74 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L9"/>
+  <dimension ref="A1:K10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="17" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="15" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="13" customWidth="1" min="9" max="9"/>
-    <col width="18" customWidth="1" min="10" max="10"/>
-    <col width="8" customWidth="1" min="11" max="11"/>
-    <col width="13" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="8" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>location</t>
+          <t>site_slug</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>datacenter</t>
+          <t>parent_location_slug</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>datacenter_slug</t>
+          <t>datahall</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>datahall</t>
+          <t>datahall_slug</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>datahall_slug</t>
+          <t>rack</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>rack</t>
+          <t>rack_u_height</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>rack_u_height</t>
+          <t>rack_width</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>rack_width</t>
+          <t>rack_status</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>rack_status</t>
+          <t>rack_form_factor</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>rack_form_factor</t>
+          <t>tenant</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>tenant</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
@@ -499,338 +493,407 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Lab Region</t>
+          <t>lab</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>LAB1</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr"/>
+          <t>lab1</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>LAB1-DH1</t>
+        </is>
+      </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>DH1</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr"/>
+          <t>lab1-dh1</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>LAB1-DH1-R09</t>
+        </is>
+      </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>LAB1-DH1-R09</t>
+          <t>45</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>45</t>
+          <t>19</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>19</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
           <t>active</t>
         </is>
       </c>
+      <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Lab Region</t>
+          <t>missing-site</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>LAB1</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr"/>
+          <t>lab1</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>LAB1-DH1</t>
+        </is>
+      </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>DH1</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr"/>
+          <t>lab1-dh1</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>MISSING-SITE-R01</t>
+        </is>
+      </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>LAB1-R05</t>
+          <t>45</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>45</t>
+          <t>19</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>19</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
           <t>active</t>
         </is>
       </c>
+      <c r="I3" t="inlineStr"/>
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Lab Region</t>
+          <t>lab</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>LAB1</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr"/>
+          <t>missing-parent</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>LAB1-DH1</t>
+        </is>
+      </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>DH1</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr"/>
+          <t>lab1-dh1</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>MISSING-PARENT-R01</t>
+        </is>
+      </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>LAB9-DH1-R06</t>
+          <t>45</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>45</t>
+          <t>19</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>19</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
           <t>active</t>
         </is>
       </c>
+      <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Lab Region</t>
+          <t>lab</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Lab Three</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr"/>
+          <t>lab1</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>LAB1-DH3</t>
+        </is>
+      </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>DH1</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr"/>
+          <t>not a slug</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>LAB1-DH3-R01</t>
+        </is>
+      </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>LAB3-DH1-R01</t>
+          <t>45</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>45</t>
+          <t>19</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>19</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
           <t>active</t>
         </is>
       </c>
+      <c r="I5" t="inlineStr"/>
       <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Lab Region</t>
+          <t>lab</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>LAB1</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr"/>
+          <t>lab1</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>LAB1-DH1</t>
+        </is>
+      </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>DH1</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr"/>
+          <t>different-slug</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>LAB1-DH1-R10</t>
+        </is>
+      </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>LAB1-DH1-R07</t>
+          <t>45</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>forty-five</t>
+          <t>19</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>19</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
           <t>active</t>
         </is>
       </c>
+      <c r="I6" t="inlineStr"/>
       <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Lab Region</t>
+          <t>lab</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>LAB1</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr"/>
+          <t>lab1</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>LAB1-DH1</t>
+        </is>
+      </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>DH1</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr"/>
+          <t>lab1-dh1</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>LAB1-DH1-R07</t>
+        </is>
+      </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>LAB1-DH1-R09</t>
+          <t>forty-five</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>45</t>
+          <t>19</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>19</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
           <t>active</t>
         </is>
       </c>
+      <c r="I7" t="inlineStr"/>
       <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Lab Region</t>
+          <t>lab</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>LAB1</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr"/>
+          <t>lab1</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>LAB1-DH1</t>
+        </is>
+      </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>DH1</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr"/>
+          <t>lab1-dh1</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>LAB1-DH1-R09</t>
+        </is>
+      </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>LAB1-DH1-R01</t>
+          <t>45</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>19</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>19</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
           <t>active</t>
         </is>
       </c>
+      <c r="I8" t="inlineStr"/>
       <c r="J8" t="inlineStr"/>
       <c r="K8" t="inlineStr"/>
-      <c r="L8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Lab Region</t>
+          <t>lab</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>LAB1</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr"/>
+          <t>lab1</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>LAB1-DH1</t>
+        </is>
+      </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>DH1</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr"/>
+          <t>lab1-dh1</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>LAB1-DH1-R01</t>
+        </is>
+      </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>LAB1-DH1-R08</t>
+          <t>12</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>45</t>
+          <t>19</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>19</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>switched-on</t>
-        </is>
-      </c>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr"/>
       <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr"/>
-      <c r="L9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>lab</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>lab1</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>LAB1-DH1</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>lab1-dh1</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>LAB1-DH1-R08</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>switched-on</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>